<commit_message>
add BOM and gerbers
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -20,11 +20,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t xml:space="preserve">Item</t>
   </si>
   <si>
+    <t xml:space="preserve">URL</t>
+  </si>
+  <si>
     <t xml:space="preserve">Price</t>
   </si>
   <si>
@@ -35,6 +38,51 @@
   </si>
   <si>
     <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STM32G071GBU6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C529347.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100nF cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C60474.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7uF cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C23733.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TS-1088-AR02016 (pushbutton)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C720477.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PZ254V-11-04P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C2691448.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PZ254V-11-03P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcsc.com/product-detail/C2937625.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Subtotal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipping and handling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PCB</t>
   </si>
 </sst>
 </file>
@@ -44,11 +92,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -64,6 +113,25 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -108,8 +176,32 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -236,32 +328,205 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.75"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.66"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="19.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18.49"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="n">
+        <f aca="false">C2*E2</f>
+        <v>1.65</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>100</v>
+      </c>
+      <c r="F3" s="1" t="n">
+        <f aca="false">C3*E3</f>
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="1" t="n">
+        <v>0.0059</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F4" s="1" t="n">
+        <f aca="false">C4*E4</f>
+        <v>0.295</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="n">
+        <v>0.0558</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1" t="n">
+        <f aca="false">C5*E5</f>
+        <v>0.558</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>0.0254</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="F6" s="1" t="n">
+        <f aca="false">C6*E6</f>
+        <v>0.508</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>0.0186</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>50</v>
+      </c>
+      <c r="F7" s="1" t="n">
+        <f aca="false">C7*E7</f>
+        <v>0.93</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <f aca="false">ROUNDUP(SUM(F2:F7),2)</f>
+        <v>4.06</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="1" t="n">
+        <f aca="false">8.72+3</f>
+        <v>11.72</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1" t="n">
+        <v>5.22</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <f aca="false">ROUNDUP(SUM(4.06+11.72)*1.0825,2)</f>
+        <v>17.09</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" display="https://www.lcsc.com/product-detail/C529347.html"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://www.lcsc.com/product-detail/C60474.html"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://www.lcsc.com/product-detail/C23733.html"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://www.lcsc.com/product-detail/C720477.html"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://www.lcsc.com/product-detail/C2691448.html"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://www.lcsc.com/product-detail/C2937625.html"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>